<commit_message>
Restore India E20 roadmap news item
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-03.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-03.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,88 +505,88 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="110.35" customHeight="1" s="2">
+    <row r="2" ht="165.35" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>印度已提前完成全国汽油E20掺混推广，BIEPA主席Pushpinder Singh建议未来5年把E30作为基础燃料，并推动灵活燃料汽车普及。E30路线会扩大燃料乙醇需求；若增量由甘蔗汁、B重糖蜜或糖浆满足，糖厂可结晶成糖的蔗糖量会减少，印度食糖供应预期下降，因此利多原糖。来源：ChiniMandi（https://www.chinimandi.com/the-road-beyond-e20-biepa-president-pushpinder-singh-on-indias-ethanol-future/）</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>利多：印度从E20迈向未来5年E30将扩大燃料乙醇需求；若增量使用甘蔗汁、B重糖蜜或糖浆制醇，会减少可结晶成糖的蔗糖量并压低食糖供应预期，从而支撑原糖价格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110.35" customHeight="1" s="2">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>泰国</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>泰国气象局预报（2026-08-03），乌隆他尼、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="118.05" customHeight="1" s="2">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4" ht="118.05" customHeight="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="180" customHeight="1" s="2">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>菲律宾糖业部门预警并加强红条软介壳虫防治，虫害已扩散至22%的甘蔗面积。虫害覆盖面积扩大将降低受害地块单产和可入榨糖料，若防治不及时会下调后续食糖产量预期，利多糖价。来源：ChiniMandi（https://news.google.com/rss/articles/CBMitgFBVV95cUxOZDB1Y283dEVuZjNJSXRhM3ZsekU0WmhNQ3NFQjRGQ1BPY1ZrMlNyd1Q1Y1EtbHNTYXdjMWEyVXhwTVJveS05VVAySmZDU2R6WkN6LVJBQmI4bDB4V2dxMzJsQWxWOFBQZzdYWUU0YW9RSW9rZ2c4RkxmY3dkSHY2bTk1eWFwQXRQZkY4UDRrdHVuTXF1a3g1TTltbExrb1VIMFpEYmNibldDXzZva0xaelh2NldTUQ?oc=5）</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>利多：红条软介壳虫扩散至22%的甘蔗面积会减少可收获糖料，并削弱后续食糖产量预期，从而支撑糖价。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="180" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>巴基斯坦</t>
+          <t>菲律宾</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>巴基斯坦糖厂协会（PSMA）要求政府批准出口58.5万吨剩余食糖。若出口获批，巴基斯坦国内库存压力将下降、国内可流通糖源减少，本地糖价受到支撑；但出口增加会补充国际市场供应。来源：UrduPoint（https://news.google.com/rss/articles/CBMimwFBVV95cUxPeFN4VWF3cG9PbHdnZDEyLWstc0ZfSzhzM0RaQzB4MExscEFObGx6MWc0MURfT3lJOVg4NkJxaWZSTnY1ckZGRlluZWR4c1I5Z0RyeFVkV2lITEdCOXc5eVNJSjdGMzVMZFEzVUtMOVZ4THlxUmVVQUlSbXZnUUxJUDFoMTB1cHRmc3JOY0dIb0o1clptMVU2RFNQdw?oc=5）</t>
+          <t>菲律宾糖业部门预警并加强红条软介壳虫防治，虫害已扩散至22%的甘蔗面积。虫害覆盖面积扩大将降低受害地块单产和可入榨糖料，若防治不及时会下调后续食糖产量预期，利多糖价。来源：ChiniMandi（https://news.google.com/rss/articles/CBMitgFBVV95cUxOZDB1Y283dEVuZjNJSXRhM3ZsekU0WmhNQ3NFQjRGQ1BPY1ZrMlNyd1Q1Y1EtbHNTYXdjMWEyVXhwTVJveS05VVAySmZDU2R6WkN6LVJBQmI4bDB4V2dxMzJsQWxWOFBQZzdYWUU0YW9RSW9rZ2c4RkxmY3dkSHY2bTk1eWFwQXRQZkY4UDRrdHVuTXF1a3g1TTltbExrb1VIMFpEYmNibldDXzZva0xaelh2NldTUQ?oc=5）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>中性：出口58.5万吨剩余食糖将减少巴基斯坦国内可流通糖源并支撑本地糖价，同时增加国际市场供应，内外盘影响相互抵消。</t>
+          <t>利多：红条软介壳虫扩散至22%的甘蔗面积会减少可收获糖料，并削弱后续食糖产量预期，从而支撑糖价。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="180" customHeight="1" s="2">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>菲律宾</t>
+          <t>巴基斯坦</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>菲律宾糖业监管署（SRA）公布数据，菲律宾原糖产量下降10.98%。产量下降会减少国内可售原糖供应，在进口补充不足时支撑菲律宾国内糖价，因此利多当地糖价。来源：Newswav（https://news.google.com/rss/articles/CBMiigFBVV95cUxNbURDSWtacnV1R2ZBVFUyczRnQ0JhclBpZlBRdkV6NFZ2VTZkcm5zUUkzdV9CQVpuLWViTjlsaE5iQUlWTE9iR0M3VFNNUnVmSTZwX1pMVGNnc0lDWXVHWWR3MU9GX0MtR25UTXFNNGRqTmR0Y3VEOVRrZTgxeF9mdmF6Qkg0akZRdGc?oc=5）</t>
+          <t>巴基斯坦糖厂协会（PSMA）要求政府批准出口58.5万吨剩余食糖。若出口获批，巴基斯坦国内库存压力将下降、国内可流通糖源减少，本地糖价受到支撑；但出口增加会补充国际市场供应。来源：UrduPoint（https://news.google.com/rss/articles/CBMimwFBVV95cUxPeFN4VWF3cG9PbHdnZDEyLWstc0ZfSzhzM0RaQzB4MExscEFObGx6MWc0MURfT3lJOVg4NkJxaWZSTnY1ckZGRlluZWR4c1I5Z0RyeFVkV2lITEdCOXc5eVNJSjdGMzVMZFEzVUtMOVZ4THlxUmVVQUlSbXZnUUxJUDFoMTB1cHRmc3JOY0dIb0o1clptMVU2RFNQdw?oc=5）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>利多：菲律宾原糖产量下降10.98%会减少国内可售糖源，若进口没有同步补充，将支撑当地糖价。</t>
+          <t>中性：出口58.5万吨剩余食糖将减少巴基斯坦国内可流通糖源并支撑本地糖价，同时增加国际市场供应，内外盘影响相互抵消。</t>
         </is>
       </c>
     </row>
@@ -598,10 +598,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>菲律宾糖业监管署（SRA）公布数据，菲律宾原糖产量下降10.98%。产量下降会减少国内可售原糖供应，在进口补充不足时支撑菲律宾国内糖价，因此利多当地糖价。来源：Newswav（https://news.google.com/rss/articles/CBMiigFBVV95cUxNbURDSWtacnV1R2ZBVFUyczRnQ0JhclBpZlBRdkV6NFZ2VTZkcm5zUUkzdV9CQVpuLWViTjlsaE5iQUlWTE9iR0M3VFNNUnVmSTZwX1pMVGNnc0lDWXVHWWR3MU9GX0MtR25UTXFNNGRqTmR0Y3VEOVRrZTgxeF9mdmF6Qkg0akZRdGc?oc=5）</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>利多：菲律宾原糖产量下降10.98%会减少国内可售糖源，若进口没有同步补充，将支撑当地糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="180" customHeight="1" s="2">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>菲律宾棉兰老岛蔗农组织预警，甘蔗病虫害已扩散至4个省。病虫害扩大将影响甘蔗生长和可收获糖料，若防控不及时，后续食糖产量预期会下调。来源：Inquirer.net（https://news.google.com/rss/articles/CBMirAFBVV95cUxQeWN2OWhuejVsRDFEZDVsUHc3Z0YwZHlNWmVpY1JaWV9LczFtb0tvUDFMVzJLVVJZa3M0Ml8zSWMxRUFYMkxSUV94SjRFa1lCQjZqYlF2dnA4ZF9mS2dRVV9kbXNHXzhKRnBqMkEtR1FadWlZVzhvZFRyODBhRXdxdFpYVlhmSElVYkJadm5PeHhZQjFiMVRBXzBKTTBWVl9CSnhISTFhX1dGNGcy0gGyAUFVX3lxTE9XdVdFQ3JWWEFicjRCYWlBSHRGTnVmUk4zS0xIWlJHdE9RaHdBbENqcnVxZGs5aGpjekV1RC1DYkJxVXprUVphd1dqR2t0ckVqdHh1NFZVV3lfZFAzc3BUa3ptcmdsMDJ3WHhRWVQ4ZUVuVkdXc0V1TkhneEpZUFN4U1NGOFVyR040dTZsTGQyejRVbXpYS0FXUHNWY3FzN0M4c1dpYXRNLUtMU1pQbWVFdkE?oc=5）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>利多：病虫害扩散会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
         </is>

</xml_diff>